<commit_message>
Add high-return quant fund sheets to screen workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WPorLsjsM2SQ8NtThS8EDA
</commit_message>
<xml_diff>
--- a/fund_research/quant_fund_screen.xlsx
+++ b/fund_research/quant_fund_screen.xlsx
@@ -10,6 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入选清单" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部量化候选(153)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方法说明" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高收益档(量化,按全期年化)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高收益(历史不足4年)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高收益(名称含智能等非量化)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +426,6 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1581,8 +1583,6 @@
       <c r="AC9" s="1" t="n">
         <v>-0.06419999999999999</v>
       </c>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
       <c r="AF9" s="1" t="inlineStr"/>
       <c r="AG9" s="1" t="inlineStr"/>
       <c r="AH9" t="n">
@@ -1856,7 +1856,6 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -2070,7 +2069,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>002943</t>
@@ -2178,10 +2176,8 @@
       <c r="AH2" t="n">
         <v>0.9526</v>
       </c>
-      <c r="AI2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>000006</t>
@@ -2293,10 +2289,8 @@
       <c r="AH3" t="n">
         <v>0.9176</v>
       </c>
-      <c r="AI3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>005616</t>
@@ -2404,10 +2398,8 @@
       <c r="AH4" t="n">
         <v>0.8928</v>
       </c>
-      <c r="AI4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>014668</t>
@@ -2511,10 +2503,8 @@
       <c r="AH5" t="n">
         <v>0.8754999999999999</v>
       </c>
-      <c r="AI5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>002561</t>
@@ -2626,10 +2616,8 @@
       <c r="AH6" t="n">
         <v>0.8588</v>
       </c>
-      <c r="AI6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>005399</t>
@@ -2741,10 +2729,8 @@
       <c r="AH7" t="n">
         <v>0.8565</v>
       </c>
-      <c r="AI7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>005960</t>
@@ -2852,10 +2838,8 @@
       <c r="AH8" t="n">
         <v>0.8484</v>
       </c>
-      <c r="AI8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>007685</t>
@@ -2963,10 +2947,8 @@
       <c r="AH9" t="n">
         <v>0.8431</v>
       </c>
-      <c r="AI9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>005635</t>
@@ -3074,10 +3056,8 @@
       <c r="AH10" t="n">
         <v>0.831</v>
       </c>
-      <c r="AI10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>001990</t>
@@ -3189,10 +3169,8 @@
       <c r="AH11" t="n">
         <v>0.8193</v>
       </c>
-      <c r="AI11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>005632</t>
@@ -3300,10 +3278,8 @@
       <c r="AH12" t="n">
         <v>0.8</v>
       </c>
-      <c r="AI12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>005457</t>
@@ -3319,7 +3295,6 @@
           <t>普通股票型</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
         <v>8.5</v>
       </c>
@@ -3407,10 +3382,8 @@
       <c r="AH13" t="n">
         <v>0.7984</v>
       </c>
-      <c r="AI13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>001244</t>
@@ -3522,10 +3495,8 @@
       <c r="AH14" t="n">
         <v>0.7977</v>
       </c>
-      <c r="AI14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>010779</t>
@@ -3637,10 +3608,8 @@
       <c r="AH15" t="n">
         <v>0.7931</v>
       </c>
-      <c r="AI15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>007808</t>
@@ -3752,10 +3721,8 @@
       <c r="AH16" t="n">
         <v>0.784</v>
       </c>
-      <c r="AI16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>000172</t>
@@ -3850,17 +3817,13 @@
       <c r="AC17" s="1" t="n">
         <v>-0.248</v>
       </c>
-      <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
       <c r="AF17" s="1" t="inlineStr"/>
       <c r="AG17" s="1" t="inlineStr"/>
       <c r="AH17" t="n">
         <v>0.782</v>
       </c>
-      <c r="AI17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>007527</t>
@@ -3972,10 +3935,8 @@
       <c r="AH18" t="n">
         <v>0.768</v>
       </c>
-      <c r="AI18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>005443</t>
@@ -4070,17 +4031,13 @@
       <c r="AC19" s="1" t="n">
         <v>-0.2762</v>
       </c>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
       <c r="AF19" s="1" t="inlineStr"/>
       <c r="AG19" s="1" t="inlineStr"/>
       <c r="AH19" t="n">
         <v>0.7608</v>
       </c>
-      <c r="AI19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>000877</t>
@@ -4175,17 +4132,13 @@
       <c r="AC20" s="1" t="n">
         <v>-0.2454</v>
       </c>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr"/>
       <c r="AF20" s="1" t="inlineStr"/>
       <c r="AG20" s="1" t="inlineStr"/>
       <c r="AH20" t="n">
         <v>0.7588</v>
       </c>
-      <c r="AI20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>006648</t>
@@ -4293,10 +4246,8 @@
       <c r="AH21" t="n">
         <v>0.7565</v>
       </c>
-      <c r="AI21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>004716</t>
@@ -4404,10 +4355,8 @@
       <c r="AH22" t="n">
         <v>0.752</v>
       </c>
-      <c r="AI22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>080005</t>
@@ -4502,17 +4451,13 @@
       <c r="AC23" s="1" t="n">
         <v>-0.1994</v>
       </c>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
       <c r="AF23" s="1" t="inlineStr"/>
       <c r="AG23" s="1" t="inlineStr"/>
       <c r="AH23" t="n">
         <v>0.7484</v>
       </c>
-      <c r="AI23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>005055</t>
@@ -4620,10 +4565,8 @@
       <c r="AH24" t="n">
         <v>0.7402</v>
       </c>
-      <c r="AI24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>001637</t>
@@ -4731,10 +4674,8 @@
       <c r="AH25" t="n">
         <v>0.7386</v>
       </c>
-      <c r="AI25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>002449</t>
@@ -4842,10 +4783,8 @@
       <c r="AH26" t="n">
         <v>0.7366</v>
       </c>
-      <c r="AI26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>481017</t>
@@ -4957,10 +4896,8 @@
       <c r="AH27" t="n">
         <v>0.7294</v>
       </c>
-      <c r="AI27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>002179</t>
@@ -5072,10 +5009,8 @@
       <c r="AH28" t="n">
         <v>0.7229</v>
       </c>
-      <c r="AI28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>007137</t>
@@ -5170,17 +5105,13 @@
       <c r="AC29" s="1" t="n">
         <v>-0.2616</v>
       </c>
-      <c r="AD29" t="inlineStr"/>
-      <c r="AE29" t="inlineStr"/>
       <c r="AF29" s="1" t="inlineStr"/>
       <c r="AG29" s="1" t="inlineStr"/>
       <c r="AH29" t="n">
         <v>0.7225</v>
       </c>
-      <c r="AI29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>005005</t>
@@ -5292,10 +5223,8 @@
       <c r="AH30" t="n">
         <v>0.7219</v>
       </c>
-      <c r="AI30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>002210</t>
@@ -5390,17 +5319,13 @@
       <c r="AC31" s="1" t="n">
         <v>-0.2397</v>
       </c>
-      <c r="AD31" t="inlineStr"/>
-      <c r="AE31" t="inlineStr"/>
       <c r="AF31" s="1" t="inlineStr"/>
       <c r="AG31" s="1" t="inlineStr"/>
       <c r="AH31" t="n">
         <v>0.7196</v>
       </c>
-      <c r="AI31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>460009</t>
@@ -5508,10 +5433,8 @@
       <c r="AH32" t="n">
         <v>0.7023</v>
       </c>
-      <c r="AI32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
           <t>001974</t>
@@ -5619,10 +5542,8 @@
       <c r="AH33" t="n">
         <v>0.6993</v>
       </c>
-      <c r="AI33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
           <t>007903</t>
@@ -5734,10 +5655,8 @@
       <c r="AH34" t="n">
         <v>0.6974</v>
       </c>
-      <c r="AI34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
           <t>014135</t>
@@ -5828,17 +5747,13 @@
       <c r="AC35" s="1" t="n">
         <v>-0.09669999999999999</v>
       </c>
-      <c r="AD35" t="inlineStr"/>
-      <c r="AE35" t="inlineStr"/>
       <c r="AF35" s="1" t="inlineStr"/>
       <c r="AG35" s="1" t="inlineStr"/>
       <c r="AH35" t="n">
         <v>0.6912</v>
       </c>
-      <c r="AI35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
           <t>005126</t>
@@ -5950,10 +5865,8 @@
       <c r="AH36" t="n">
         <v>0.6859</v>
       </c>
-      <c r="AI36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
           <t>005225</t>
@@ -6048,17 +5961,13 @@
       <c r="AC37" s="1" t="n">
         <v>-0.2285</v>
       </c>
-      <c r="AD37" t="inlineStr"/>
-      <c r="AE37" t="inlineStr"/>
       <c r="AF37" s="1" t="inlineStr"/>
       <c r="AG37" s="1" t="inlineStr"/>
       <c r="AH37" t="n">
         <v>0.6837</v>
       </c>
-      <c r="AI37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>006022</t>
@@ -6096,7 +6005,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
         <v>0.2042</v>
       </c>
@@ -6151,17 +6059,13 @@
       <c r="AC38" s="1" t="n">
         <v>-0.1737</v>
       </c>
-      <c r="AD38" t="inlineStr"/>
-      <c r="AE38" t="inlineStr"/>
       <c r="AF38" s="1" t="inlineStr"/>
       <c r="AG38" s="1" t="inlineStr"/>
       <c r="AH38" t="n">
         <v>0.6804</v>
       </c>
-      <c r="AI38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t>000609</t>
@@ -6273,10 +6177,8 @@
       <c r="AH39" t="n">
         <v>0.668</v>
       </c>
-      <c r="AI39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>015006</t>
@@ -6292,7 +6194,6 @@
           <t>偏股混合型</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
         <v>4.5</v>
       </c>
@@ -6380,10 +6281,8 @@
       <c r="AH40" t="n">
         <v>0.6582</v>
       </c>
-      <c r="AI40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>001980</t>
@@ -6491,10 +6390,8 @@
       <c r="AH41" t="n">
         <v>0.6451</v>
       </c>
-      <c r="AI41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>004641</t>
@@ -6606,10 +6503,8 @@
       <c r="AH42" t="n">
         <v>0.6307</v>
       </c>
-      <c r="AI42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>000199</t>
@@ -6704,17 +6599,13 @@
       <c r="AC43" s="1" t="n">
         <v>-0.2876</v>
       </c>
-      <c r="AD43" t="inlineStr"/>
-      <c r="AE43" t="inlineStr"/>
       <c r="AF43" s="1" t="inlineStr"/>
       <c r="AG43" s="1" t="inlineStr"/>
       <c r="AH43" t="n">
         <v>0.6294</v>
       </c>
-      <c r="AI43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>014691</t>
@@ -6818,10 +6709,8 @@
       <c r="AH44" t="n">
         <v>0.6225000000000001</v>
       </c>
-      <c r="AI44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>002270</t>
@@ -6929,10 +6818,8 @@
       <c r="AH45" t="n">
         <v>0.6183</v>
       </c>
-      <c r="AI45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>006336</t>
@@ -7027,17 +6914,13 @@
       <c r="AC46" s="1" t="n">
         <v>-0.2203</v>
       </c>
-      <c r="AD46" t="inlineStr"/>
-      <c r="AE46" t="inlineStr"/>
       <c r="AF46" s="1" t="inlineStr"/>
       <c r="AG46" s="1" t="inlineStr"/>
       <c r="AH46" t="n">
         <v>0.6133999999999999</v>
       </c>
-      <c r="AI46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>519975</t>
@@ -7145,10 +7028,8 @@
       <c r="AH47" t="n">
         <v>0.6078</v>
       </c>
-      <c r="AI47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>630015</t>
@@ -7260,10 +7141,8 @@
       <c r="AH48" t="n">
         <v>0.602</v>
       </c>
-      <c r="AI48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>005075</t>
@@ -7375,10 +7254,8 @@
       <c r="AH49" t="n">
         <v>0.5997</v>
       </c>
-      <c r="AI49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
           <t>002952</t>
@@ -7486,10 +7363,8 @@
       <c r="AH50" t="n">
         <v>0.5585</v>
       </c>
-      <c r="AI50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
           <t>005269</t>
@@ -7597,10 +7472,8 @@
       <c r="AH51" t="n">
         <v>0.5575</v>
       </c>
-      <c r="AI51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
           <t>000978</t>
@@ -7708,10 +7581,8 @@
       <c r="AH52" t="n">
         <v>0.552</v>
       </c>
-      <c r="AI52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
           <t>519965</t>
@@ -7823,10 +7694,8 @@
       <c r="AH53" t="n">
         <v>0.55</v>
       </c>
-      <c r="AI53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
           <t>002300</t>
@@ -7864,7 +7733,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="n">
         <v>0.1507</v>
       </c>
@@ -7932,10 +7800,8 @@
       <c r="AH54" t="n">
         <v>0.5376</v>
       </c>
-      <c r="AI54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
           <t>004394</t>
@@ -8043,10 +7909,8 @@
       <c r="AH55" t="n">
         <v>0.535</v>
       </c>
-      <c r="AI55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
           <t>519983</t>
@@ -8158,10 +8022,8 @@
       <c r="AH56" t="n">
         <v>0.5324</v>
       </c>
-      <c r="AI56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
           <t>014187</t>
@@ -8269,10 +8131,8 @@
       <c r="AH57" t="n">
         <v>0.5258</v>
       </c>
-      <c r="AI57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
           <t>008077</t>
@@ -8367,17 +8227,13 @@
       <c r="AC58" s="1" t="n">
         <v>-0.1588</v>
       </c>
-      <c r="AD58" t="inlineStr"/>
-      <c r="AE58" t="inlineStr"/>
       <c r="AF58" s="1" t="inlineStr"/>
       <c r="AG58" s="1" t="inlineStr"/>
       <c r="AH58" t="n">
         <v>0.5242</v>
       </c>
-      <c r="AI58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
           <t>002216</t>
@@ -8485,10 +8341,8 @@
       <c r="AH59" t="n">
         <v>0.5203</v>
       </c>
-      <c r="AI59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
           <t>002562</t>
@@ -8526,7 +8380,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="n">
         <v>0.1673</v>
       </c>
@@ -8581,17 +8434,13 @@
       <c r="AC60" s="1" t="n">
         <v>-0.256</v>
       </c>
-      <c r="AD60" t="inlineStr"/>
-      <c r="AE60" t="inlineStr"/>
       <c r="AF60" s="1" t="inlineStr"/>
       <c r="AG60" s="1" t="inlineStr"/>
       <c r="AH60" t="n">
         <v>0.5196</v>
       </c>
-      <c r="AI60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
           <t>003069</t>
@@ -8703,10 +8552,8 @@
       <c r="AH61" t="n">
         <v>0.517</v>
       </c>
-      <c r="AI61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
           <t>001789</t>
@@ -8801,17 +8648,13 @@
       <c r="AC62" s="1" t="n">
         <v>-0.2303</v>
       </c>
-      <c r="AD62" t="inlineStr"/>
-      <c r="AE62" t="inlineStr"/>
       <c r="AF62" s="1" t="inlineStr"/>
       <c r="AG62" s="1" t="inlineStr"/>
       <c r="AH62" t="n">
         <v>0.5137</v>
       </c>
-      <c r="AI62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
           <t>002495</t>
@@ -8849,7 +8692,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
       <c r="L63" t="n">
         <v>0.16</v>
       </c>
@@ -8904,17 +8746,13 @@
       <c r="AC63" s="1" t="n">
         <v>-0.2792</v>
       </c>
-      <c r="AD63" t="inlineStr"/>
-      <c r="AE63" t="inlineStr"/>
       <c r="AF63" s="1" t="inlineStr"/>
       <c r="AG63" s="1" t="inlineStr"/>
       <c r="AH63" t="n">
         <v>0.5095</v>
       </c>
-      <c r="AI63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
           <t>002862</t>
@@ -9022,10 +8860,8 @@
       <c r="AH64" t="n">
         <v>0.5069</v>
       </c>
-      <c r="AI64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
           <t>166107</t>
@@ -9041,7 +8877,6 @@
           <t>偏股混合型</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="n">
         <v>6.8</v>
       </c>
@@ -9129,10 +8964,8 @@
       <c r="AH65" t="n">
         <v>0.502</v>
       </c>
-      <c r="AI65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
           <t>011824</t>
@@ -9240,10 +9073,8 @@
       <c r="AH66" t="n">
         <v>0.4984</v>
       </c>
-      <c r="AI66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
           <t>233009</t>
@@ -9351,10 +9182,8 @@
       <c r="AH67" t="n">
         <v>0.4984</v>
       </c>
-      <c r="AI67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
           <t>002983</t>
@@ -9466,10 +9295,8 @@
       <c r="AH68" t="n">
         <v>0.4971</v>
       </c>
-      <c r="AI68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
           <t>003241</t>
@@ -9507,7 +9334,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
       <c r="L69" t="n">
         <v>0.1103</v>
       </c>
@@ -9562,17 +9388,13 @@
       <c r="AC69" s="1" t="n">
         <v>-0.2477</v>
       </c>
-      <c r="AD69" t="inlineStr"/>
-      <c r="AE69" t="inlineStr"/>
       <c r="AF69" s="1" t="inlineStr"/>
       <c r="AG69" s="1" t="inlineStr"/>
       <c r="AH69" t="n">
         <v>0.4958</v>
       </c>
-      <c r="AI69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
           <t>005120</t>
@@ -9680,10 +9502,8 @@
       <c r="AH70" t="n">
         <v>0.4918</v>
       </c>
-      <c r="AI70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
           <t>012297</t>
@@ -9778,17 +9598,13 @@
       <c r="AC71" s="1" t="n">
         <v>-0.1367</v>
       </c>
-      <c r="AD71" t="inlineStr"/>
-      <c r="AE71" t="inlineStr"/>
       <c r="AF71" s="1" t="inlineStr"/>
       <c r="AG71" s="1" t="inlineStr"/>
       <c r="AH71" t="n">
         <v>0.4905</v>
       </c>
-      <c r="AI71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
           <t>005189</t>
@@ -9826,7 +9642,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
       <c r="L72" t="n">
         <v>0.1367</v>
       </c>
@@ -9894,10 +9709,8 @@
       <c r="AH72" t="n">
         <v>0.482</v>
       </c>
-      <c r="AI72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
           <t>014995</t>
@@ -9913,7 +9726,6 @@
           <t>偏股混合型</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="n">
         <v>4.5</v>
       </c>
@@ -9984,17 +9796,13 @@
       <c r="AC73" s="1" t="n">
         <v>-0.1057</v>
       </c>
-      <c r="AD73" t="inlineStr"/>
-      <c r="AE73" t="inlineStr"/>
       <c r="AF73" s="1" t="inlineStr"/>
       <c r="AG73" s="1" t="inlineStr"/>
       <c r="AH73" t="n">
         <v>0.4722</v>
       </c>
-      <c r="AI73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
           <t>005258</t>
@@ -10102,10 +9910,8 @@
       <c r="AH74" t="n">
         <v>0.4621</v>
       </c>
-      <c r="AI74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
           <t>005650</t>
@@ -10217,10 +10023,8 @@
       <c r="AH75" t="n">
         <v>0.4595</v>
       </c>
-      <c r="AI75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
           <t>014701</t>
@@ -10328,10 +10132,8 @@
       <c r="AH76" t="n">
         <v>0.4578</v>
       </c>
-      <c r="AI76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
           <t>005437</t>
@@ -10439,10 +10241,8 @@
       <c r="AH77" t="n">
         <v>0.4471</v>
       </c>
-      <c r="AI77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
           <t>070017</t>
@@ -10550,10 +10350,8 @@
       <c r="AH78" t="n">
         <v>0.4461</v>
       </c>
-      <c r="AI78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
           <t>006106</t>
@@ -10665,10 +10463,8 @@
       <c r="AH79" t="n">
         <v>0.4412</v>
       </c>
-      <c r="AI79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
           <t>001017</t>
@@ -10706,7 +10502,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
       <c r="L80" t="n">
         <v>0.1539</v>
       </c>
@@ -10774,10 +10569,8 @@
       <c r="AH80" t="n">
         <v>0.4408</v>
       </c>
-      <c r="AI80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
           <t>519929</t>
@@ -10872,17 +10665,13 @@
       <c r="AC81" s="1" t="n">
         <v>-0.3428</v>
       </c>
-      <c r="AD81" t="inlineStr"/>
-      <c r="AE81" t="inlineStr"/>
       <c r="AF81" s="1" t="inlineStr"/>
       <c r="AG81" s="1" t="inlineStr"/>
       <c r="AH81" t="n">
         <v>0.4389</v>
       </c>
-      <c r="AI81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
           <t>011410</t>
@@ -10977,17 +10766,13 @@
       <c r="AC82" s="1" t="n">
         <v>-0.1862</v>
       </c>
-      <c r="AD82" t="inlineStr"/>
-      <c r="AE82" t="inlineStr"/>
       <c r="AF82" s="1" t="inlineStr"/>
       <c r="AG82" s="1" t="inlineStr"/>
       <c r="AH82" t="n">
         <v>0.4373</v>
       </c>
-      <c r="AI82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
           <t>005707</t>
@@ -11095,10 +10880,8 @@
       <c r="AH83" t="n">
         <v>0.434</v>
       </c>
-      <c r="AI83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
           <t>005082</t>
@@ -11210,10 +10993,8 @@
       <c r="AH84" t="n">
         <v>0.4294</v>
       </c>
-      <c r="AI84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
           <t>360001</t>
@@ -11308,17 +11089,13 @@
       <c r="AC85" s="1" t="n">
         <v>-0.6371</v>
       </c>
-      <c r="AD85" t="inlineStr"/>
-      <c r="AE85" t="inlineStr"/>
       <c r="AF85" s="1" t="inlineStr"/>
       <c r="AG85" s="1" t="inlineStr"/>
       <c r="AH85" t="n">
         <v>0.4281</v>
       </c>
-      <c r="AI85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
           <t>007775</t>
@@ -11426,10 +11203,8 @@
       <c r="AH86" t="n">
         <v>0.4268</v>
       </c>
-      <c r="AI86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
           <t>011107</t>
@@ -11537,10 +11312,8 @@
       <c r="AH87" t="n">
         <v>0.417</v>
       </c>
-      <c r="AI87" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
           <t>006267</t>
@@ -11578,7 +11351,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
       <c r="L88" t="n">
         <v>0.1159</v>
       </c>
@@ -11650,10 +11422,8 @@
       <c r="AH88" t="n">
         <v>0.4095</v>
       </c>
-      <c r="AI88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
           <t>003717</t>
@@ -11761,10 +11531,8 @@
       <c r="AH89" t="n">
         <v>0.4078</v>
       </c>
-      <c r="AI89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
           <t>010137</t>
@@ -11872,10 +11640,8 @@
       <c r="AH90" t="n">
         <v>0.4003</v>
       </c>
-      <c r="AI90" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
           <t>005865</t>
@@ -11913,7 +11679,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" t="n">
         <v>0.0318</v>
       </c>
@@ -11981,10 +11746,8 @@
       <c r="AH91" t="n">
         <v>0.3974</v>
       </c>
-      <c r="AI91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
           <t>010303</t>
@@ -12092,10 +11855,8 @@
       <c r="AH92" t="n">
         <v>0.3922</v>
       </c>
-      <c r="AI92" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
           <t>004925</t>
@@ -12133,7 +11894,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" t="n">
         <v>0.1199</v>
       </c>
@@ -12188,17 +11948,13 @@
       <c r="AC93" s="1" t="n">
         <v>-0.3207</v>
       </c>
-      <c r="AD93" t="inlineStr"/>
-      <c r="AE93" t="inlineStr"/>
       <c r="AF93" s="1" t="inlineStr"/>
       <c r="AG93" s="1" t="inlineStr"/>
       <c r="AH93" t="n">
         <v>0.385</v>
       </c>
-      <c r="AI93" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
           <t>000646</t>
@@ -12310,10 +12066,8 @@
       <c r="AH94" t="n">
         <v>0.3732</v>
       </c>
-      <c r="AI94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr"/>
       <c r="B95" t="inlineStr">
         <is>
           <t>007853</t>
@@ -12425,10 +12179,8 @@
       <c r="AH95" t="n">
         <v>0.365</v>
       </c>
-      <c r="AI95" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr">
         <is>
           <t>003147</t>
@@ -12540,10 +12292,8 @@
       <c r="AH96" t="n">
         <v>0.3637</v>
       </c>
-      <c r="AI96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr"/>
       <c r="B97" t="inlineStr">
         <is>
           <t>010690</t>
@@ -12655,10 +12405,8 @@
       <c r="AH97" t="n">
         <v>0.3627</v>
       </c>
-      <c r="AI97" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr"/>
       <c r="B98" t="inlineStr">
         <is>
           <t>006449</t>
@@ -12696,7 +12444,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="n">
         <v>0.1</v>
       </c>
@@ -12764,10 +12511,8 @@
       <c r="AH98" t="n">
         <v>0.3624</v>
       </c>
-      <c r="AI98" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr"/>
       <c r="B99" t="inlineStr">
         <is>
           <t>005037</t>
@@ -12805,7 +12550,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="n">
         <v>0.09909999999999999</v>
       </c>
@@ -12860,17 +12604,13 @@
       <c r="AC99" s="1" t="n">
         <v>-0.3186</v>
       </c>
-      <c r="AD99" t="inlineStr"/>
-      <c r="AE99" t="inlineStr"/>
       <c r="AF99" s="1" t="inlineStr"/>
       <c r="AG99" s="1" t="inlineStr"/>
       <c r="AH99" t="n">
         <v>0.3595</v>
       </c>
-      <c r="AI99" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr"/>
       <c r="B100" t="inlineStr">
         <is>
           <t>167702</t>
@@ -12908,7 +12648,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="n">
         <v>0.0934</v>
       </c>
@@ -12949,7 +12688,7 @@
         <v>-0.4206</v>
       </c>
       <c r="Y100" s="1" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z100" s="1" t="n">
         <v>-0.3116</v>
@@ -12980,10 +12719,8 @@
       <c r="AH100" t="n">
         <v>0.3582</v>
       </c>
-      <c r="AI100" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr"/>
       <c r="B101" t="inlineStr">
         <is>
           <t>009557</t>
@@ -13095,10 +12832,8 @@
       <c r="AH101" t="n">
         <v>0.3513</v>
       </c>
-      <c r="AI101" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
       <c r="B102" t="inlineStr">
         <is>
           <t>009992</t>
@@ -13206,10 +12941,8 @@
       <c r="AH102" t="n">
         <v>0.3392</v>
       </c>
-      <c r="AI102" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr"/>
       <c r="B103" t="inlineStr">
         <is>
           <t>001421</t>
@@ -13317,10 +13050,8 @@
       <c r="AH103" t="n">
         <v>0.3369</v>
       </c>
-      <c r="AI103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr"/>
       <c r="B104" t="inlineStr">
         <is>
           <t>001291</t>
@@ -13358,7 +13089,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="n">
         <v>0.0618</v>
       </c>
@@ -13430,10 +13160,8 @@
       <c r="AH104" t="n">
         <v>0.3343</v>
       </c>
-      <c r="AI104" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr"/>
       <c r="B105" t="inlineStr">
         <is>
           <t>005235</t>
@@ -13471,7 +13199,6 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="n">
         <v>0.0911</v>
       </c>
@@ -13526,17 +13253,13 @@
       <c r="AC105" s="1" t="n">
         <v>-0.2137</v>
       </c>
-      <c r="AD105" t="inlineStr"/>
-      <c r="AE105" t="inlineStr"/>
       <c r="AF105" s="1" t="inlineStr"/>
       <c r="AG105" s="1" t="inlineStr"/>
       <c r="AH105" t="n">
         <v>0.3271</v>
       </c>
-      <c r="AI105" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr"/>
       <c r="B106" t="inlineStr">
         <is>
           <t>011224</t>
@@ -13631,17 +13354,13 @@
       <c r="AC106" s="1" t="n">
         <v>-0.1577</v>
       </c>
-      <c r="AD106" t="inlineStr"/>
-      <c r="AE106" t="inlineStr"/>
       <c r="AF106" s="1" t="inlineStr"/>
       <c r="AG106" s="1" t="inlineStr"/>
       <c r="AH106" t="n">
         <v>0.3258</v>
       </c>
-      <c r="AI106" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr"/>
       <c r="B107" t="inlineStr">
         <is>
           <t>398041</t>
@@ -13679,7 +13398,6 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" t="n">
         <v>0.0526</v>
       </c>
@@ -13747,10 +13465,8 @@
       <c r="AH107" t="n">
         <v>0.3258</v>
       </c>
-      <c r="AI107" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr"/>
       <c r="B108" t="inlineStr">
         <is>
           <t>166109</t>
@@ -13858,10 +13574,8 @@
       <c r="AH108" t="n">
         <v>0.3101</v>
       </c>
-      <c r="AI108" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr"/>
       <c r="B109" t="inlineStr">
         <is>
           <t>001219</t>
@@ -13973,10 +13687,8 @@
       <c r="AH109" t="n">
         <v>0.3049</v>
       </c>
-      <c r="AI109" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr"/>
       <c r="B110" t="inlineStr">
         <is>
           <t>012878</t>
@@ -14071,17 +13783,13 @@
       <c r="AC110" s="1" t="n">
         <v>-0.1675</v>
       </c>
-      <c r="AD110" t="inlineStr"/>
-      <c r="AE110" t="inlineStr"/>
       <c r="AF110" s="1" t="inlineStr"/>
       <c r="AG110" s="1" t="inlineStr"/>
       <c r="AH110" t="n">
         <v>0.3</v>
       </c>
-      <c r="AI110" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr"/>
       <c r="B111" t="inlineStr">
         <is>
           <t>005947</t>
@@ -14119,7 +13827,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
       <c r="L111" t="n">
         <v>0.0818</v>
       </c>
@@ -14187,10 +13894,8 @@
       <c r="AH111" t="n">
         <v>0.2967</v>
       </c>
-      <c r="AI111" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr"/>
       <c r="B112" t="inlineStr">
         <is>
           <t>009043</t>
@@ -14228,7 +13933,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
       <c r="L112" t="n">
         <v>0.0415</v>
       </c>
@@ -14296,10 +14000,8 @@
       <c r="AH112" t="n">
         <v>0.282</v>
       </c>
-      <c r="AI112" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr"/>
       <c r="B113" t="inlineStr">
         <is>
           <t>001897</t>
@@ -14337,7 +14039,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
       <c r="L113" t="n">
         <v>0.06660000000000001</v>
       </c>
@@ -14392,17 +14093,13 @@
       <c r="AC113" s="1" t="n">
         <v>-0.2272</v>
       </c>
-      <c r="AD113" t="inlineStr"/>
-      <c r="AE113" t="inlineStr"/>
       <c r="AF113" s="1" t="inlineStr"/>
       <c r="AG113" s="1" t="inlineStr"/>
       <c r="AH113" t="n">
         <v>0.266</v>
       </c>
-      <c r="AI113" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr"/>
       <c r="B114" t="inlineStr">
         <is>
           <t>011934</t>
@@ -14497,17 +14194,13 @@
       <c r="AC114" s="1" t="n">
         <v>-0.1252</v>
       </c>
-      <c r="AD114" t="inlineStr"/>
-      <c r="AE114" t="inlineStr"/>
       <c r="AF114" s="1" t="inlineStr"/>
       <c r="AG114" s="1" t="inlineStr"/>
       <c r="AH114" t="n">
         <v>0.265</v>
       </c>
-      <c r="AI114" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr"/>
       <c r="B115" t="inlineStr">
         <is>
           <t>007354</t>
@@ -14602,17 +14295,13 @@
       <c r="AC115" s="1" t="n">
         <v>-0.2187</v>
       </c>
-      <c r="AD115" t="inlineStr"/>
-      <c r="AE115" t="inlineStr"/>
       <c r="AF115" s="1" t="inlineStr"/>
       <c r="AG115" s="1" t="inlineStr"/>
       <c r="AH115" t="n">
         <v>0.2621</v>
       </c>
-      <c r="AI115" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr"/>
       <c r="B116" t="inlineStr">
         <is>
           <t>014139</t>
@@ -14720,10 +14409,8 @@
       <c r="AH116" t="n">
         <v>0.2608</v>
       </c>
-      <c r="AI116" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr"/>
       <c r="B117" t="inlineStr">
         <is>
           <t>009246</t>
@@ -14761,7 +14448,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr"/>
       <c r="L117" t="n">
         <v>0.0429</v>
       </c>
@@ -14829,10 +14515,8 @@
       <c r="AH117" t="n">
         <v>0.2556</v>
       </c>
-      <c r="AI117" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
       <c r="B118" t="inlineStr">
         <is>
           <t>005237</t>
@@ -14870,7 +14554,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr"/>
       <c r="L118" t="n">
         <v>0.0389</v>
       </c>
@@ -14925,17 +14608,13 @@
       <c r="AC118" s="1" t="n">
         <v>-0.2631</v>
       </c>
-      <c r="AD118" t="inlineStr"/>
-      <c r="AE118" t="inlineStr"/>
       <c r="AF118" s="1" t="inlineStr"/>
       <c r="AG118" s="1" t="inlineStr"/>
       <c r="AH118" t="n">
         <v>0.2549</v>
       </c>
-      <c r="AI118" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr"/>
       <c r="B119" t="inlineStr">
         <is>
           <t>011589</t>
@@ -14973,7 +14652,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr"/>
       <c r="L119" t="n">
         <v>-0.1797</v>
       </c>
@@ -15037,10 +14715,8 @@
       <c r="AH119" t="n">
         <v>0.25</v>
       </c>
-      <c r="AI119" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
       <c r="B120" t="inlineStr">
         <is>
           <t>014020</t>
@@ -15148,10 +14824,8 @@
       <c r="AH120" t="n">
         <v>0.2444</v>
       </c>
-      <c r="AI120" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr"/>
       <c r="B121" t="inlineStr">
         <is>
           <t>014062</t>
@@ -15242,17 +14916,13 @@
       <c r="AC121" s="1" t="n">
         <v>-0.2607</v>
       </c>
-      <c r="AD121" t="inlineStr"/>
-      <c r="AE121" t="inlineStr"/>
       <c r="AF121" s="1" t="inlineStr"/>
       <c r="AG121" s="1" t="inlineStr"/>
       <c r="AH121" t="n">
         <v>0.2353</v>
       </c>
-      <c r="AI121" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
       <c r="B122" t="inlineStr">
         <is>
           <t>014171</t>
@@ -15343,17 +15013,13 @@
       <c r="AC122" s="1" t="n">
         <v>-0.1787</v>
       </c>
-      <c r="AD122" t="inlineStr"/>
-      <c r="AE122" t="inlineStr"/>
       <c r="AF122" s="1" t="inlineStr"/>
       <c r="AG122" s="1" t="inlineStr"/>
       <c r="AH122" t="n">
         <v>0.2275</v>
       </c>
-      <c r="AI122" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
       <c r="B123" t="inlineStr">
         <is>
           <t>013918</t>
@@ -15457,10 +15123,8 @@
       <c r="AH123" t="n">
         <v>0.2235</v>
       </c>
-      <c r="AI123" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
       <c r="B124" t="inlineStr">
         <is>
           <t>233015</t>
@@ -15498,7 +15162,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr"/>
       <c r="L124" t="n">
         <v>0.0449</v>
       </c>
@@ -15570,10 +15233,8 @@
       <c r="AH124" t="n">
         <v>0.2023</v>
       </c>
-      <c r="AI124" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
       <c r="B125" t="inlineStr">
         <is>
           <t>001143</t>
@@ -15611,7 +15272,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr"/>
       <c r="L125" t="n">
         <v>0.0369</v>
       </c>
@@ -15683,10 +15343,8 @@
       <c r="AH125" t="n">
         <v>0.182</v>
       </c>
-      <c r="AI125" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
       <c r="B126" t="inlineStr">
         <is>
           <t>009840</t>
@@ -15724,7 +15382,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr"/>
       <c r="L126" t="n">
         <v>-0.0281</v>
       </c>
@@ -15792,10 +15449,8 @@
       <c r="AH126" t="n">
         <v>0.1794</v>
       </c>
-      <c r="AI126" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
       <c r="B127" t="inlineStr">
         <is>
           <t>004209</t>
@@ -15833,7 +15488,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr"/>
       <c r="L127" t="n">
         <v>0.0254</v>
       </c>
@@ -15901,10 +15555,8 @@
       <c r="AH127" t="n">
         <v>0.1752</v>
       </c>
-      <c r="AI127" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr"/>
       <c r="B128" t="inlineStr">
         <is>
           <t>012977</t>
@@ -15920,7 +15572,6 @@
           <t>偏股混合型</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="n">
         <v>5.1</v>
       </c>
@@ -15938,7 +15589,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr"/>
       <c r="L128" t="n">
         <v>-0.0593</v>
       </c>
@@ -16010,10 +15660,8 @@
       <c r="AH128" t="n">
         <v>0.1647</v>
       </c>
-      <c r="AI128" t="inlineStr"/>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr"/>
       <c r="B129" t="inlineStr">
         <is>
           <t>010120</t>
@@ -16051,7 +15699,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr"/>
       <c r="L129" t="n">
         <v>-0.0285</v>
       </c>
@@ -16119,10 +15766,8 @@
       <c r="AH129" t="n">
         <v>0.1641</v>
       </c>
-      <c r="AI129" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr"/>
       <c r="B130" t="inlineStr">
         <is>
           <t>006785</t>
@@ -16160,7 +15805,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr"/>
       <c r="L130" t="n">
         <v>0.0162</v>
       </c>
@@ -16228,10 +15872,8 @@
       <c r="AH130" t="n">
         <v>0.1304</v>
       </c>
-      <c r="AI130" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr"/>
       <c r="B131" t="inlineStr">
         <is>
           <t>010293</t>
@@ -16269,7 +15911,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr"/>
       <c r="L131" t="n">
         <v>-0.0444</v>
       </c>
@@ -16341,10 +15982,8 @@
       <c r="AH131" t="n">
         <v>0.1258</v>
       </c>
-      <c r="AI131" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr"/>
       <c r="B132" t="inlineStr">
         <is>
           <t>008353</t>
@@ -16382,7 +16021,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr"/>
       <c r="L132" t="n">
         <v>-0.0239</v>
       </c>
@@ -16450,10 +16088,8 @@
       <c r="AH132" t="n">
         <v>0.1203</v>
       </c>
-      <c r="AI132" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr"/>
       <c r="B133" t="inlineStr">
         <is>
           <t>009874</t>
@@ -16491,7 +16127,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr"/>
       <c r="L133" t="n">
         <v>-0.1367</v>
       </c>
@@ -16559,10 +16194,8 @@
       <c r="AH133" t="n">
         <v>0.1193</v>
       </c>
-      <c r="AI133" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr"/>
       <c r="B134" t="inlineStr">
         <is>
           <t>011500</t>
@@ -16670,10 +16303,8 @@
       <c r="AH134" t="n">
         <v>0.1114</v>
       </c>
-      <c r="AI134" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr"/>
       <c r="B135" t="inlineStr">
         <is>
           <t>580007</t>
@@ -16711,7 +16342,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr"/>
       <c r="L135" t="n">
         <v>-0.0086</v>
       </c>
@@ -16779,10 +16409,8 @@
       <c r="AH135" t="n">
         <v>0.1</v>
       </c>
-      <c r="AI135" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr"/>
       <c r="B136" t="inlineStr">
         <is>
           <t>010801</t>
@@ -16820,7 +16448,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr"/>
       <c r="L136" t="n">
         <v>-0.195</v>
       </c>
@@ -16875,17 +16502,13 @@
       <c r="AC136" s="1" t="n">
         <v>-0.1833</v>
       </c>
-      <c r="AD136" t="inlineStr"/>
-      <c r="AE136" t="inlineStr"/>
       <c r="AF136" s="1" t="inlineStr"/>
       <c r="AG136" s="1" t="inlineStr"/>
       <c r="AH136" t="n">
         <v>0.09710000000000001</v>
       </c>
-      <c r="AI136" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr"/>
       <c r="B137" t="inlineStr">
         <is>
           <t>002919</t>
@@ -16923,7 +16546,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr"/>
       <c r="L137" t="n">
         <v>-0.0269</v>
       </c>
@@ -16995,10 +16617,8 @@
       <c r="AH137" t="n">
         <v>0.0951</v>
       </c>
-      <c r="AI137" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr"/>
       <c r="B138" t="inlineStr">
         <is>
           <t>010296</t>
@@ -17036,7 +16656,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K138" t="inlineStr"/>
       <c r="L138" t="n">
         <v>-0.0411</v>
       </c>
@@ -17108,10 +16727,8 @@
       <c r="AH138" t="n">
         <v>0.0853</v>
       </c>
-      <c r="AI138" t="inlineStr"/>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr"/>
       <c r="B139" t="inlineStr">
         <is>
           <t>006926</t>
@@ -17149,7 +16766,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr"/>
       <c r="L139" t="n">
         <v>-0.0835</v>
       </c>
@@ -17217,10 +16833,8 @@
       <c r="AH139" t="n">
         <v>0.0837</v>
       </c>
-      <c r="AI139" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr"/>
       <c r="B140" t="inlineStr">
         <is>
           <t>004805</t>
@@ -17258,7 +16872,6 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr"/>
       <c r="L140" t="n">
         <v>-0.0268</v>
       </c>
@@ -17326,10 +16939,8 @@
       <c r="AH140" t="n">
         <v>0.0742</v>
       </c>
-      <c r="AI140" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr"/>
       <c r="B141" t="inlineStr">
         <is>
           <t>005255</t>
@@ -17367,7 +16978,6 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr"/>
       <c r="L141" t="n">
         <v>-0.073</v>
       </c>
@@ -17439,10 +17049,8 @@
       <c r="AH141" t="n">
         <v>0.0716</v>
       </c>
-      <c r="AI141" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr"/>
       <c r="B142" t="inlineStr">
         <is>
           <t>005599</t>
@@ -17480,7 +17088,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K142" t="inlineStr"/>
       <c r="L142" t="n">
         <v>-0.0481</v>
       </c>
@@ -17548,10 +17155,8 @@
       <c r="AH142" t="n">
         <v>0.06859999999999999</v>
       </c>
-      <c r="AI142" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr"/>
       <c r="B143" t="inlineStr">
         <is>
           <t>005347</t>
@@ -17589,7 +17194,6 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="K143" t="inlineStr"/>
       <c r="L143" t="n">
         <v>-0.0755</v>
       </c>
@@ -17661,10 +17265,8 @@
       <c r="AH143" t="n">
         <v>0.067</v>
       </c>
-      <c r="AI143" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr"/>
       <c r="B144" t="inlineStr">
         <is>
           <t>006877</t>
@@ -17702,7 +17304,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
       <c r="L144" t="n">
         <v>-0.1327</v>
       </c>
@@ -17770,7 +17371,6 @@
       <c r="AH144" t="n">
         <v>0.015</v>
       </c>
-      <c r="AI144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -18717,8 +18317,6 @@
       <c r="AC152" s="1" t="n">
         <v>-0.06419999999999999</v>
       </c>
-      <c r="AD152" t="inlineStr"/>
-      <c r="AE152" t="inlineStr"/>
       <c r="AF152" s="1" t="inlineStr"/>
       <c r="AG152" s="1" t="inlineStr"/>
       <c r="AH152" t="n">
@@ -19052,4 +18650,1617 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>基金名称</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>历史年数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>全期年化</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>近3年年化</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>全期最大回撤(月频)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>熊市区间收益</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>现任经理</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>现任经理任职(年)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>现任期年化</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>007685</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>华商电子行业量化股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>0.3884</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>-0.4782</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>-0.2785</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>艾定飞</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1.7796</v>
+      </c>
+      <c r="J2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>002943</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>广发多因子灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.1985</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0.1603</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>-0.3202</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>0.0187</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>杨冬</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0.4271</v>
+      </c>
+      <c r="J3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>000006</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>西部利得量化成长混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.1833</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0.1403</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>-0.3654</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>-0.1847</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>盛丰衍</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>5.6947</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>0.0824</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>014805</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>国金量化精选混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.1745</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0.1511</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>-0.2414</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>0.0507</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>马芳</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>4.5202</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>0.1748</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>006195</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>国金量化多因子股票型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0.1618</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0.1622</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>-0.2379</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>0.1349</v>
+      </c>
+      <c r="J6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>007808</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>华银量化优选灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0.2566</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>-0.4609</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>-0.3522</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>程敏</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>7.0171</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>0.154</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>008251</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>汇安宜创量化精选混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0.1408</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>0.2123</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>-0.3397</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>-0.285</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>柳预才</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>5.0568</v>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>0.0769</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>001917</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>招商量化精选股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0.1394</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>0.1816</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>-0.3358</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>0.1969</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>王平</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>7.0363</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>0.2083</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>000609</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>华商新量化灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>0.2177</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>-0.5143</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>-0.3884</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>邓默</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>4.2163</v>
+      </c>
+      <c r="J10" s="1" t="n">
+        <v>0.0805</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>014668</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>银华专精特新量化优选股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0.1325</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>0.2083</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>-0.2929</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>-0.2735</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>杨腾</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1.5359</v>
+      </c>
+      <c r="J11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>007527</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>融通量化多策略灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0.1296</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>0.1624</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>-0.4096</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>-0.2727</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>蔡志伟</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>3.7728</v>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>0.0953</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>005638</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>农银汇理量化智慧动力混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>0.1294</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>0.1196</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>-0.3213</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>-0.1808</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>魏刚</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>8.4983</v>
+      </c>
+      <c r="J13" s="1" t="n">
+        <v>0.1294</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>006648</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>汇安多因子混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0.1289</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>0.1918</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>-0.408</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>-0.4032</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>柳预才</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>2.3792</v>
+      </c>
+      <c r="J14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>016466</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>国泰海通量化选股混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>0.1281</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>0.1563</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>-0.2199</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>胡崇海</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>4.1013</v>
+      </c>
+      <c r="J15" s="1" t="n">
+        <v>0.1349</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>481017</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>工银瑞信基本面量化策略混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>0.1278</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>0.1717</v>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>-0.4484</v>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>-0.3251</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>张乐涛</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>4.4107</v>
+      </c>
+      <c r="J16" s="1" t="n">
+        <v>0.0728</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>006401</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>先锋量化优选灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>0.1201</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>0.1559</v>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>-0.3498</v>
+      </c>
+      <c r="G17" s="1" t="n">
+        <v>-0.1328</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>曾捷</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>3.6988</v>
+      </c>
+      <c r="J17" s="1" t="n">
+        <v>0.117</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>001990</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>中欧数据挖掘多因子灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0.1173</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>0.1797</v>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>-0.3715</v>
+      </c>
+      <c r="G18" s="1" t="n">
+        <v>-0.2564</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>曲径</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>4.9829</v>
+      </c>
+      <c r="J18" s="1" t="n">
+        <v>0.0528</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>013465</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>博时智选量化多因子股票型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>0.1163</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>0.2313</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>-0.2753</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>刘钊</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>4.8925</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>0.1135</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>000172</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>华泰柏瑞量化增强混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>0.1142</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>0.1169</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>-0.3419</v>
+      </c>
+      <c r="G20" s="1" t="n">
+        <v>-0.2737</v>
+      </c>
+      <c r="J20" s="1" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>005225</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>广发量化多因子灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0.1116</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>0.2278</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>-0.4517</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>-0.4373</v>
+      </c>
+      <c r="J21" s="1" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>基金名称</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>历史年数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>全期年化</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>近3年年化</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>全期最大回撤(月频)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>熊市区间收益</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>现任经理</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>现任经理任职(年)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>现任期年化</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>020476</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>泰康半导体量化选股股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.6728</v>
+      </c>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="n">
+        <v>-0.3239</v>
+      </c>
+      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>袁帅</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1.3224</v>
+      </c>
+      <c r="J2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>022754</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>易方达科鑫量化选股股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.5082</v>
+      </c>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="n">
+        <v>-0.2046</v>
+      </c>
+      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>包正钰</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1.7851</v>
+      </c>
+      <c r="J3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>020975</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>万家科技量化选股混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.3806</v>
+      </c>
+      <c r="E4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="n">
+        <v>-0.2229</v>
+      </c>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>尹航</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>1.9986</v>
+      </c>
+      <c r="J4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>021990</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>中加专精特新量化选股混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="E5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="n">
+        <v>-0.1384</v>
+      </c>
+      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>林沐尘</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>1.8645</v>
+      </c>
+      <c r="J5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>020698</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>国泰海通科创板量化选股股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0.3463</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr"/>
+      <c r="F6" s="1" t="n">
+        <v>-0.2971</v>
+      </c>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>胡崇海</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>2.4394</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>0.3463</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>020560</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>万家高端装备量化选股混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.2672</v>
+      </c>
+      <c r="E7" s="1" t="inlineStr"/>
+      <c r="F7" s="1" t="n">
+        <v>-0.2539</v>
+      </c>
+      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>尹航</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>2.6804</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>0.2958</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>021812</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>东兴宸泰量化选股混合发起A</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0.2642</v>
+      </c>
+      <c r="E8" s="1" t="inlineStr"/>
+      <c r="F8" s="1" t="n">
+        <v>-0.1576</v>
+      </c>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>李兵伟</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>1.9932</v>
+      </c>
+      <c r="J8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>019722</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>中银量化选股混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0.2581</v>
+      </c>
+      <c r="E9" s="1" t="inlineStr"/>
+      <c r="F9" s="1" t="n">
+        <v>-0.1743</v>
+      </c>
+      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>赵志华</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>2.2697</v>
+      </c>
+      <c r="J9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>020901</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>招商成长量化选股股票A</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0.2418</v>
+      </c>
+      <c r="E10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>王平</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>2.3162</v>
+      </c>
+      <c r="J10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>021884</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>太平量化选股混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0.2172</v>
+      </c>
+      <c r="E11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="n">
+        <v>-0.167</v>
+      </c>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>张子权</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1.9028</v>
+      </c>
+      <c r="J11" s="1" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>基金名称</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>历史年数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>全期年化</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>近3年年化</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>全期最大回撤(月频)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>熊市区间收益</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>现任经理</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>现任经理任职(年)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>现任期年化</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>005825</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>申万菱信智能驱动股票型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>0.5489000000000001</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>-0.4377</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>卜忠林</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0.5202</v>
+      </c>
+      <c r="J2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>005962</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>宝盈人工智能主题股票型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.2319</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0.3403</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>-0.543</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>-0.3419</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>叶秀贤</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0.7803</v>
+      </c>
+      <c r="J3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>005914</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>景顺长城智能生活混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.2253</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0.397</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>-0.4892</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>-0.4333</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>江山</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>1.6701</v>
+      </c>
+      <c r="J4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>006281</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>万家人工智能混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.2082</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>-0.5217000000000001</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>-0.196</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>耿嘉洲</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>4.846</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>0.0565</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>005729</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>南方人工智能主题混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0.1833</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0.1893</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>-0.4029</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>-0.2654</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>罗安安</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>7.9507</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>0.1833</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>009644</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>东方阿尔法优势产业混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.1714</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0.2966</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>-0.6287</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>-0.2663</v>
+      </c>
+      <c r="J7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>015143</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>中欧智能制造混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0.1693</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>0.3175</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>-0.3656</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>-0.2269</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>刘金辉、邵洁</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0.0219</v>
+      </c>
+      <c r="J8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>005844</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>东方人工智能主题混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0.1582</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>0.4723</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>-0.4917</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>-0.4316</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>严凯</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>5.9384</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>0.1593</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>006863</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>国联安智能制造混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>0.2388</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>-0.4683</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>-0.4683</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>高诗</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>1.306</v>
+      </c>
+      <c r="J10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>006879</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>华安智能生活混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0.1499</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>0.06469999999999999</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>-0.3618</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>-0.2124</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>胡宜斌</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>4.9336</v>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>0.0168</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 5-year annualized return ranking sheet for quant funds
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WPorLsjsM2SQ8NtThS8EDA
</commit_message>
<xml_diff>
--- a/fund_research/quant_fund_screen.xlsx
+++ b/fund_research/quant_fund_screen.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高收益档(量化,按全期年化)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高收益(历史不足4年)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高收益(名称含智能等非量化)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="近5年年化Top25" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20263,4 +20264,1049 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>基金名称</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>历史年数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>近5年年化(2021.9起)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>近5年最大回撤</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>近5年卡玛</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>近3年年化</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>全期年化</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>现任经理</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>现任经理任职(年)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>现任期年化</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>006195</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>国金量化多因子股票型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.1539</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>-0.2379</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.647</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>0.1622</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>0.1618</v>
+      </c>
+      <c r="K2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>007685</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>华商电子行业量化股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.1393</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>-0.473</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2945</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>0.3884</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>艾定飞</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1.7796</v>
+      </c>
+      <c r="K3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>001917</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>招商量化精选股票型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.1252</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>-0.1782</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.7029</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>0.1816</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>0.1394</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>王平</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>7.0363</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>0.2083</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>005443</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>国金量化多策略灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.1153</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>-0.2183</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.5281</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>0.0796</v>
+      </c>
+      <c r="K5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>519929</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>长信电子信息行业量化灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0.09180000000000001</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>-0.5125</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1791</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>0.3339</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>0.08119999999999999</v>
+      </c>
+      <c r="K6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>002449</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>民生加银量化中国灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.0854</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>-0.06759999999999999</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.2627</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>0.1115</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>0.0621</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>周帅</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>1.5797</v>
+      </c>
+      <c r="K7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>005632</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>鹏华量化先锋混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0.0815</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>-0.2453</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.3322</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>0.1761</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>0.0926</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>时赟超</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>1.692</v>
+      </c>
+      <c r="K8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>002943</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>广发多因子灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0.08019999999999999</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>-0.3202</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2503</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>0.1603</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>0.1985</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>杨冬</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0.4271</v>
+      </c>
+      <c r="K9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>002862</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>金信量化精选灵活配置混合型发起式证券投资基金</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0.0801</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>-0.4968</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1613</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>0.0823</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>孔学兵</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0.2464</v>
+      </c>
+      <c r="K10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>004641</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>万家量化睿选灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0.0774</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>-0.3519</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>0.1759</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>0.0867</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>乔亮</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>4.0821</v>
+      </c>
+      <c r="K11" s="1" t="n">
+        <v>0.1045</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>001244</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>华泰柏瑞量化智慧灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0.0774</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>-0.2515</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.3078</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>0.1845</v>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>笪篁</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>4.8925</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>0.083</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>005616</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>东方量化成长灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>0.0764</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>-0.2488</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.3069</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>0.1672</v>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>0.1062</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>王怀勋</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>1.5359</v>
+      </c>
+      <c r="K13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>005126</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>银河量化稳进混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>-0.3081</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.2335</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>0.1841</v>
+      </c>
+      <c r="H14" s="1" t="n">
+        <v>0.0736</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>罗博</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>5.3032</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>0.0713</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>008251</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>汇安宜创量化精选混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>-0.3397</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.2032</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>0.2123</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>0.1408</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>柳预才</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>5.0568</v>
+      </c>
+      <c r="K15" s="1" t="n">
+        <v>0.0769</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>005457</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>景顺长城量化小盘股票A</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>0.0669</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>-0.3467</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.1929</v>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>0.1708</v>
+      </c>
+      <c r="H16" s="1" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>黎海威</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>1.3689</v>
+      </c>
+      <c r="K16" s="1" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>010779</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>西部利得量化优选一年持有期混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>0.06660000000000001</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>-0.3739</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.1781</v>
+      </c>
+      <c r="G17" s="1" t="n">
+        <v>0.1979</v>
+      </c>
+      <c r="H17" s="1" t="n">
+        <v>0.1037</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>翟梓舰</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>2.8966</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>0.1956</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>002179</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>华安事件驱动量化策略混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>-0.412</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.1552</v>
+      </c>
+      <c r="G18" s="1" t="n">
+        <v>0.2201</v>
+      </c>
+      <c r="H18" s="1" t="n">
+        <v>0.1073</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>张序</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>3.5154</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>0.1212</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>460009</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>华泰柏瑞量化先行混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>-0.2922</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.2166</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>0.1633</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>0.0915</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>盛豪</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>1.4073</v>
+      </c>
+      <c r="K19" s="1" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>006648</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>汇安多因子混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>0.06270000000000001</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>-0.3846</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.1629</v>
+      </c>
+      <c r="G20" s="1" t="n">
+        <v>0.1918</v>
+      </c>
+      <c r="H20" s="1" t="n">
+        <v>0.1289</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>柳预才</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>2.3792</v>
+      </c>
+      <c r="K20" s="1" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>005635</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>博时量化多策略股票型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0.0616</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>-0.2538</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.2425</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>0.1433</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>0.1011</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>刘玉强</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0.7693</v>
+      </c>
+      <c r="K21" s="1" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>005960</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>博时量化价值股票型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>0.0608</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>-0.2163</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.2811</v>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>杨振建</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>0.7693</v>
+      </c>
+      <c r="K22" s="1" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>004250</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>银河量化优选混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>0.0587</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>-0.293</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.2002</v>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>0.1541</v>
+      </c>
+      <c r="H23" s="1" t="n">
+        <v>0.1092</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>罗博</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>3.1595</v>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>0.1383</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>000646</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>华润元大量化优选混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>0.0583</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>-0.3418</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.1706</v>
+      </c>
+      <c r="G24" s="1" t="n">
+        <v>0.1171</v>
+      </c>
+      <c r="H24" s="1" t="n">
+        <v>0.0573</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>李武群</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>3.1403</v>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>0.1171</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>010137</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>华泰柏瑞量化创享混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>0.0567</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>-0.4772</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.1188</v>
+      </c>
+      <c r="G25" s="1" t="n">
+        <v>0.2345</v>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>0.0617</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>凌若冰</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>1.4073</v>
+      </c>
+      <c r="K25" s="1" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>007808</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>华银量化优选灵活配置混合型证券投资基金</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>0.0555</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>-0.4609</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.1203</v>
+      </c>
+      <c r="G26" s="1" t="n">
+        <v>0.2566</v>
+      </c>
+      <c r="H26" s="1" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>程敏</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>7.0171</v>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>0.154</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>